<commit_message>
Update ETF pipeline and provider outputs
</commit_message>
<xml_diff>
--- a/providers/franklintempleton/2026-06-24/UCITS_ETF_FUNDS.xlsx
+++ b/providers/franklintempleton/2026-06-24/UCITS_ETF_FUNDS.xlsx
@@ -398,7 +398,7 @@
         <v>as of</v>
       </c>
       <c r="B3" s="1">
-        <v>46195.041666666664</v>
+        <v>46196.041666666664</v>
       </c>
     </row>
     <row r="5">
@@ -456,19 +456,19 @@
         <v>USD</v>
       </c>
       <c r="F6">
-        <v>29.91</v>
+        <v>29.11</v>
       </c>
       <c r="G6">
-        <v>7.1</v>
+        <v>6.97</v>
       </c>
       <c r="H6">
         <v>102</v>
       </c>
       <c r="I6">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="J6" t="str">
-        <v>$131.79 Million</v>
+        <v>$129.36 Million</v>
       </c>
       <c r="K6">
         <v>6</v>
@@ -494,10 +494,10 @@
         <v>USD</v>
       </c>
       <c r="F7">
-        <v>24.57</v>
+        <v>24.19</v>
       </c>
       <c r="G7">
-        <v>3.99</v>
+        <v>3.93</v>
       </c>
       <c r="H7">
         <v>1434</v>
@@ -506,7 +506,7 @@
         <v>—</v>
       </c>
       <c r="J7" t="str">
-        <v>$21.81 Million</v>
+        <v>$21.42 Million</v>
       </c>
       <c r="K7">
         <v>6</v>
@@ -532,19 +532,19 @@
         <v>USD</v>
       </c>
       <c r="F8">
-        <v>28.64</v>
+        <v>28.23</v>
       </c>
       <c r="G8">
-        <v>7.32</v>
+        <v>7.21</v>
       </c>
       <c r="H8">
         <v>222</v>
       </c>
       <c r="I8">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="J8" t="str">
-        <v>$351.64 Million</v>
+        <v>$343.30 Million</v>
       </c>
       <c r="K8">
         <v>8</v>
@@ -570,19 +570,19 @@
         <v>EUR</v>
       </c>
       <c r="F9">
-        <v>19.12</v>
+        <v>18.97</v>
       </c>
       <c r="G9">
-        <v>2.5</v>
+        <v>2.48</v>
       </c>
       <c r="H9">
         <v>475</v>
       </c>
       <c r="I9">
-        <v>2.76</v>
+        <v>2.78</v>
       </c>
       <c r="J9" t="str">
-        <v>€34.19 Million</v>
+        <v>€33.91 Million</v>
       </c>
       <c r="K9">
         <v>8</v>
@@ -608,19 +608,19 @@
         <v>USD</v>
       </c>
       <c r="F10">
-        <v>26.9</v>
+        <v>26.49</v>
       </c>
       <c r="G10">
-        <v>5.86</v>
+        <v>5.77</v>
       </c>
       <c r="H10">
         <v>212</v>
       </c>
       <c r="I10">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="J10" t="str">
-        <v>$76.62 Million</v>
+        <v>$75.49 Million</v>
       </c>
       <c r="K10">
         <v>6</v>
@@ -646,10 +646,10 @@
         <v>USD</v>
       </c>
       <c r="F11">
-        <v>15.51</v>
+        <v>15.52</v>
       </c>
       <c r="G11">
-        <v>2.12</v>
+        <v>2.11</v>
       </c>
       <c r="H11">
         <v>65</v>
@@ -658,7 +658,7 @@
         <v>—</v>
       </c>
       <c r="J11" t="str">
-        <v>$6.20 Million</v>
+        <v>$6.19 Million</v>
       </c>
       <c r="K11">
         <v>6</v>
@@ -696,7 +696,7 @@
         <v>—</v>
       </c>
       <c r="J12" t="str">
-        <v>$5.69 Million</v>
+        <v>$5.57 Million</v>
       </c>
       <c r="K12">
         <v>6</v>
@@ -734,7 +734,7 @@
         <v>1.68</v>
       </c>
       <c r="J13" t="str">
-        <v>$2.69 Million</v>
+        <v>$2.72 Million</v>
       </c>
       <c r="K13">
         <v>8</v>
@@ -760,19 +760,19 @@
         <v>USD</v>
       </c>
       <c r="F14">
-        <v>23.65</v>
+        <v>23.37</v>
       </c>
       <c r="G14">
-        <v>3.92</v>
+        <v>3.87</v>
       </c>
       <c r="H14">
         <v>851</v>
       </c>
       <c r="I14">
-        <v>1.63</v>
+        <v>1.65</v>
       </c>
       <c r="J14" t="str">
-        <v>$14.27 Million</v>
+        <v>$14.08 Million</v>
       </c>
       <c r="K14">
         <v>8</v>
@@ -798,10 +798,10 @@
         <v>USD</v>
       </c>
       <c r="F15">
-        <v>29.54</v>
+        <v>28.79</v>
       </c>
       <c r="G15">
-        <v>5.18</v>
+        <v>4.92</v>
       </c>
       <c r="H15">
         <v>77</v>
@@ -810,7 +810,7 @@
         <v>0.01</v>
       </c>
       <c r="J15" t="str">
-        <v>$22.61 Million</v>
+        <v>$22.02 Million</v>
       </c>
       <c r="K15">
         <v>6</v>
@@ -836,10 +836,10 @@
         <v>USD</v>
       </c>
       <c r="F16">
-        <v>27</v>
+        <v>26.6</v>
       </c>
       <c r="G16">
-        <v>5.19</v>
+        <v>5.12</v>
       </c>
       <c r="H16">
         <v>278</v>
@@ -848,7 +848,7 @@
         <v>—</v>
       </c>
       <c r="J16" t="str">
-        <v>$5.02 Million</v>
+        <v>$4.94 Million</v>
       </c>
       <c r="K16">
         <v>6</v>
@@ -874,10 +874,10 @@
         <v>USD</v>
       </c>
       <c r="F17">
-        <v>27</v>
+        <v>26.6</v>
       </c>
       <c r="G17">
-        <v>5.19</v>
+        <v>5.12</v>
       </c>
       <c r="H17">
         <v>278</v>
@@ -886,7 +886,7 @@
         <v>—</v>
       </c>
       <c r="J17" t="str">
-        <v>$5.02 Million</v>
+        <v>$4.94 Million</v>
       </c>
       <c r="K17">
         <v>6</v>
@@ -912,10 +912,10 @@
         <v>USD</v>
       </c>
       <c r="F18">
-        <v>22.29</v>
+        <v>20.12</v>
       </c>
       <c r="G18">
-        <v>2.6</v>
+        <v>2.35</v>
       </c>
       <c r="H18">
         <v>157</v>
@@ -924,7 +924,7 @@
         <v>—</v>
       </c>
       <c r="J18" t="str">
-        <v>$5.27 Billion</v>
+        <v>$4.75 Billion</v>
       </c>
       <c r="K18">
         <v>6</v>
@@ -950,19 +950,19 @@
         <v>USD</v>
       </c>
       <c r="F19">
-        <v>26.52</v>
+        <v>26.15</v>
       </c>
       <c r="G19">
-        <v>5.85</v>
+        <v>5.77</v>
       </c>
       <c r="H19">
         <v>204</v>
       </c>
       <c r="I19">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="J19" t="str">
-        <v>$2.94 Million</v>
+        <v>$2.91 Million</v>
       </c>
       <c r="K19">
         <v>6</v>
@@ -988,10 +988,10 @@
         <v>USD</v>
       </c>
       <c r="F20">
-        <v>10.81</v>
+        <v>10.82</v>
       </c>
       <c r="G20">
-        <v>1.65</v>
+        <v>1.66</v>
       </c>
       <c r="H20">
         <v>76</v>
@@ -1000,7 +1000,7 @@
         <v>—</v>
       </c>
       <c r="J20" t="str">
-        <v>$148.26 Million</v>
+        <v>$148.03 Million</v>
       </c>
       <c r="K20">
         <v>6</v>
@@ -1026,16 +1026,16 @@
         <v>USD</v>
       </c>
       <c r="F21">
-        <v>17.33</v>
+        <v>17.39</v>
       </c>
       <c r="G21">
-        <v>2.35</v>
+        <v>2.36</v>
       </c>
       <c r="H21">
         <v>76</v>
       </c>
       <c r="I21">
-        <v>1.55</v>
+        <v>1.54</v>
       </c>
       <c r="J21" t="str">
         <v>$1.56 Million</v>
@@ -1064,19 +1064,19 @@
         <v>USD</v>
       </c>
       <c r="F22">
-        <v>11.36</v>
+        <v>11.18</v>
       </c>
       <c r="G22">
-        <v>1.59</v>
+        <v>1.56</v>
       </c>
       <c r="H22">
         <v>315</v>
       </c>
       <c r="I22">
-        <v>4.06</v>
+        <v>4.08</v>
       </c>
       <c r="J22" t="str">
-        <v>$88.37 Million</v>
+        <v>$86.69 Million</v>
       </c>
       <c r="K22">
         <v>6</v>
@@ -1102,7 +1102,7 @@
         <v>EUR</v>
       </c>
       <c r="F23">
-        <v>14.92</v>
+        <v>14.91</v>
       </c>
       <c r="G23">
         <v>2.52</v>
@@ -1114,7 +1114,7 @@
         <v>4.66</v>
       </c>
       <c r="J23" t="str">
-        <v>€555.75 Million</v>
+        <v>€554.89 Million</v>
       </c>
       <c r="K23">
         <v>6</v>
@@ -1140,7 +1140,7 @@
         <v>EUR</v>
       </c>
       <c r="F24">
-        <v>14.92</v>
+        <v>14.91</v>
       </c>
       <c r="G24">
         <v>2.52</v>
@@ -1152,7 +1152,7 @@
         <v>4.66</v>
       </c>
       <c r="J24" t="str">
-        <v>€555.75 Million</v>
+        <v>€554.89 Million</v>
       </c>
       <c r="K24">
         <v>6</v>
@@ -1178,10 +1178,10 @@
         <v>USD</v>
       </c>
       <c r="F25">
-        <v>26.31</v>
+        <v>26.02</v>
       </c>
       <c r="G25">
-        <v>3.5</v>
+        <v>3.46</v>
       </c>
       <c r="H25">
         <v>279</v>
@@ -1190,7 +1190,7 @@
         <v>—</v>
       </c>
       <c r="J25" t="str">
-        <v>$2.06 Billion</v>
+        <v>$2.04 Billion</v>
       </c>
       <c r="K25">
         <v>6</v>
@@ -1216,19 +1216,19 @@
         <v>USD</v>
       </c>
       <c r="F26">
-        <v>26.26</v>
+        <v>25.7</v>
       </c>
       <c r="G26">
-        <v>4.66</v>
+        <v>4.56</v>
       </c>
       <c r="H26">
         <v>648</v>
       </c>
       <c r="I26">
-        <v>1.34</v>
+        <v>1.37</v>
       </c>
       <c r="J26" t="str">
-        <v>$188.34 Million</v>
+        <v>$183.79 Million</v>
       </c>
       <c r="K26">
         <v>8</v>
@@ -1254,19 +1254,19 @@
         <v>USD</v>
       </c>
       <c r="F27">
-        <v>20.47</v>
+        <v>20.3</v>
       </c>
       <c r="G27">
-        <v>3.1</v>
+        <v>3.07</v>
       </c>
       <c r="H27">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="I27" t="str">
         <v>—</v>
       </c>
       <c r="J27" t="str">
-        <v>$7.24 Million</v>
+        <v>$7.16 Million</v>
       </c>
       <c r="K27">
         <v>6</v>
@@ -1292,19 +1292,19 @@
         <v>USD</v>
       </c>
       <c r="F28">
-        <v>17.64</v>
+        <v>17.42</v>
       </c>
       <c r="G28">
-        <v>2.37</v>
+        <v>2.34</v>
       </c>
       <c r="H28">
-        <v>1598</v>
+        <v>1597</v>
       </c>
       <c r="I28">
-        <v>2.19</v>
+        <v>2.22</v>
       </c>
       <c r="J28" t="str">
-        <v>$13.70 Million</v>
+        <v>$13.48 Million</v>
       </c>
       <c r="K28">
         <v>6</v>
@@ -1330,19 +1330,19 @@
         <v>USD</v>
       </c>
       <c r="F29">
-        <v>17.64</v>
+        <v>17.42</v>
       </c>
       <c r="G29">
-        <v>2.37</v>
+        <v>2.34</v>
       </c>
       <c r="H29">
-        <v>1598</v>
+        <v>1597</v>
       </c>
       <c r="I29">
-        <v>2.19</v>
+        <v>2.22</v>
       </c>
       <c r="J29" t="str">
-        <v>$13.70 Million</v>
+        <v>$13.48 Million</v>
       </c>
       <c r="K29">
         <v>6</v>
@@ -1368,19 +1368,19 @@
         <v>USD</v>
       </c>
       <c r="F30">
-        <v>37.77</v>
+        <v>36.4</v>
       </c>
       <c r="G30">
-        <v>14.26</v>
+        <v>13.74</v>
       </c>
       <c r="H30">
         <v>74</v>
       </c>
       <c r="I30">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="J30" t="str">
-        <v>$2.88 Million</v>
+        <v>$2.77 Million</v>
       </c>
       <c r="K30">
         <v>6</v>
@@ -1406,10 +1406,10 @@
         <v>USD</v>
       </c>
       <c r="F31">
-        <v>26.52</v>
+        <v>26.15</v>
       </c>
       <c r="G31">
-        <v>5.39</v>
+        <v>5.31</v>
       </c>
       <c r="H31" t="str">
         <v>—</v>
@@ -1418,7 +1418,7 @@
         <v>—</v>
       </c>
       <c r="J31" t="str">
-        <v>$5.41 Million</v>
+        <v>$5.34 Million</v>
       </c>
       <c r="K31">
         <v>8</v>
@@ -1447,7 +1447,7 @@
         <v>—</v>
       </c>
       <c r="G32">
-        <v>3.25</v>
+        <v>3.26</v>
       </c>
       <c r="H32" t="str">
         <v>—</v>
@@ -1456,7 +1456,7 @@
         <v>—</v>
       </c>
       <c r="J32" t="str">
-        <v>$24.80 Million</v>
+        <v>$24.83 Million</v>
       </c>
       <c r="K32">
         <v>6</v>
@@ -1482,19 +1482,19 @@
         <v>USD</v>
       </c>
       <c r="F33">
-        <v>26.83</v>
+        <v>26.5</v>
       </c>
       <c r="G33">
-        <v>5.56</v>
+        <v>5.49</v>
       </c>
       <c r="H33">
         <v>412</v>
       </c>
       <c r="I33">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="J33" t="str">
-        <v>$4.22 Million</v>
+        <v>$4.16 Million</v>
       </c>
       <c r="K33">
         <v>8</v>
@@ -1520,10 +1520,10 @@
         <v>USD</v>
       </c>
       <c r="F34">
-        <v>12.63</v>
+        <v>12.32</v>
       </c>
       <c r="G34">
-        <v>1.41</v>
+        <v>1.37</v>
       </c>
       <c r="H34">
         <v>1135</v>
@@ -1532,7 +1532,7 @@
         <v>—</v>
       </c>
       <c r="J34" t="str">
-        <v>$1.58 Billion</v>
+        <v>$1.54 Billion</v>
       </c>
       <c r="K34">
         <v>6</v>
@@ -1558,10 +1558,10 @@
         <v>USD</v>
       </c>
       <c r="F35">
-        <v>32.47</v>
+        <v>32.06</v>
       </c>
       <c r="G35">
-        <v>4.75</v>
+        <v>4.69</v>
       </c>
       <c r="H35">
         <v>133</v>
@@ -1570,7 +1570,7 @@
         <v>—</v>
       </c>
       <c r="J35" t="str">
-        <v>$578.60 Million</v>
+        <v>$570.34 Million</v>
       </c>
       <c r="K35">
         <v>6</v>
@@ -1596,10 +1596,10 @@
         <v>USD</v>
       </c>
       <c r="F36">
-        <v>17.37</v>
+        <v>17.42</v>
       </c>
       <c r="G36">
-        <v>3.54</v>
+        <v>3.55</v>
       </c>
       <c r="H36">
         <v>23</v>
@@ -1608,7 +1608,7 @@
         <v>1.3</v>
       </c>
       <c r="J36" t="str">
-        <v>$1.39 Million</v>
+        <v>$1.40 Million</v>
       </c>
       <c r="K36">
         <v>6</v>
@@ -1634,19 +1634,19 @@
         <v>USD</v>
       </c>
       <c r="F37">
-        <v>17.89</v>
+        <v>17.45</v>
       </c>
       <c r="G37">
-        <v>2.19</v>
+        <v>2.13</v>
       </c>
       <c r="H37">
         <v>132</v>
       </c>
       <c r="I37">
-        <v>1.37</v>
+        <v>1.41</v>
       </c>
       <c r="J37" t="str">
-        <v>$9.43 Million</v>
+        <v>$9.19 Million</v>
       </c>
       <c r="K37">
         <v>8</v>
@@ -1672,19 +1672,19 @@
         <v>USD</v>
       </c>
       <c r="F38">
-        <v>24.6</v>
+        <v>23.57</v>
       </c>
       <c r="G38">
-        <v>3.35</v>
+        <v>3.2</v>
       </c>
       <c r="H38">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="I38" t="str">
         <v>—</v>
       </c>
       <c r="J38" t="str">
-        <v>$580.10 Million</v>
+        <v>$554.95 Million</v>
       </c>
       <c r="K38">
         <v>6</v>
@@ -1722,7 +1722,7 @@
         <v>2.6</v>
       </c>
       <c r="J39" t="str">
-        <v>$5.48 Million</v>
+        <v>$5.45 Million</v>
       </c>
       <c r="K39">
         <v>8</v>
@@ -1748,19 +1748,19 @@
         <v>USD</v>
       </c>
       <c r="F40">
-        <v>19.27</v>
+        <v>19.2</v>
       </c>
       <c r="G40">
-        <v>4.01</v>
+        <v>3.99</v>
       </c>
       <c r="H40">
         <v>102</v>
       </c>
       <c r="I40">
-        <v>3.1</v>
+        <v>3.11</v>
       </c>
       <c r="J40" t="str">
-        <v>$116.29 Million</v>
+        <v>$115.58 Million</v>
       </c>
       <c r="K40">
         <v>6</v>
@@ -1786,19 +1786,19 @@
         <v>USD</v>
       </c>
       <c r="F41">
-        <v>19.27</v>
+        <v>19.2</v>
       </c>
       <c r="G41">
-        <v>4.01</v>
+        <v>3.99</v>
       </c>
       <c r="H41">
         <v>102</v>
       </c>
       <c r="I41">
-        <v>3.1</v>
+        <v>3.11</v>
       </c>
       <c r="J41" t="str">
-        <v>$116.29 Million</v>
+        <v>$115.58 Million</v>
       </c>
       <c r="K41">
         <v>6</v>
@@ -1824,10 +1824,10 @@
         <v>JPY</v>
       </c>
       <c r="F42">
-        <v>19.68</v>
+        <v>19.11</v>
       </c>
       <c r="G42">
-        <v>1.96</v>
+        <v>1.9</v>
       </c>
       <c r="H42">
         <v>473</v>
@@ -1836,7 +1836,7 @@
         <v>—</v>
       </c>
       <c r="J42" t="str">
-        <v>¥1.85 Billion</v>
+        <v>¥1.80 Billion</v>
       </c>
       <c r="K42">
         <v>6</v>
@@ -1862,19 +1862,19 @@
         <v>USD</v>
       </c>
       <c r="F43">
-        <v>21.76</v>
+        <v>21.07</v>
       </c>
       <c r="G43">
-        <v>3.7</v>
+        <v>3.58</v>
       </c>
       <c r="H43">
         <v>328</v>
       </c>
       <c r="I43">
-        <v>1.65</v>
+        <v>1.7</v>
       </c>
       <c r="J43" t="str">
-        <v>$9.26 Million</v>
+        <v>$8.93 Million</v>
       </c>
       <c r="K43">
         <v>8</v>
@@ -2017,7 +2017,7 @@
         <v>as of</v>
       </c>
       <c r="B3" s="1">
-        <v>46195.041666666664</v>
+        <v>46196.041666666664</v>
       </c>
     </row>
     <row r="5">
@@ -2075,19 +2075,19 @@
         <v>EUR</v>
       </c>
       <c r="F6">
-        <v>5.51</v>
+        <v>5.53</v>
       </c>
       <c r="G6">
-        <v>3.57</v>
+        <v>3.55</v>
       </c>
       <c r="H6" t="str">
         <v>A</v>
       </c>
       <c r="I6">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J6" t="str">
-        <v>€216.80 Million</v>
+        <v>€217.31 Million</v>
       </c>
       <c r="K6">
         <v>9</v>
@@ -2113,10 +2113,10 @@
         <v>EUR</v>
       </c>
       <c r="F7">
-        <v>7.36</v>
+        <v>7.37</v>
       </c>
       <c r="G7">
-        <v>3.2</v>
+        <v>3.18</v>
       </c>
       <c r="H7" t="str">
         <v>AA</v>
@@ -2125,7 +2125,7 @@
         <v>28</v>
       </c>
       <c r="J7" t="str">
-        <v>€100.97 Million</v>
+        <v>€101.20 Million</v>
       </c>
       <c r="K7">
         <v>9</v>
@@ -2151,10 +2151,10 @@
         <v>USD</v>
       </c>
       <c r="F8">
-        <v>6.85</v>
+        <v>6.84</v>
       </c>
       <c r="G8">
-        <v>5.11</v>
+        <v>5.13</v>
       </c>
       <c r="H8" t="str">
         <v>BBB-</v>
@@ -2163,7 +2163,7 @@
         <v>65</v>
       </c>
       <c r="J8" t="str">
-        <v>$68.82 Million</v>
+        <v>$68.66 Million</v>
       </c>
       <c r="K8">
         <v>8</v>
@@ -2192,7 +2192,7 @@
         <v>0.32</v>
       </c>
       <c r="G9">
-        <v>3.81</v>
+        <v>3.8</v>
       </c>
       <c r="H9" t="str">
         <v>AA+</v>
@@ -2201,7 +2201,7 @@
         <v>43</v>
       </c>
       <c r="J9" t="str">
-        <v>$104.12 Million</v>
+        <v>$103.07 Million</v>
       </c>
       <c r="K9">
         <v>6</v>
@@ -2227,19 +2227,19 @@
         <v>EUR</v>
       </c>
       <c r="F10">
-        <v>4.19</v>
+        <v>4.21</v>
       </c>
       <c r="G10">
-        <v>3.48</v>
+        <v>3.46</v>
       </c>
       <c r="H10" t="str">
         <v>A-</v>
       </c>
       <c r="I10">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J10" t="str">
-        <v>€108.01 Million</v>
+        <v>€108.15 Million</v>
       </c>
       <c r="K10">
         <v>8</v>
@@ -2265,10 +2265,10 @@
         <v>USD</v>
       </c>
       <c r="F11">
-        <v>6.73</v>
+        <v>6.74</v>
       </c>
       <c r="G11">
-        <v>5.21</v>
+        <v>5.2</v>
       </c>
       <c r="H11" t="str">
         <v>A-</v>
@@ -2277,7 +2277,7 @@
         <v>154</v>
       </c>
       <c r="J11" t="str">
-        <v>$29.68 Million</v>
+        <v>$29.72 Million</v>
       </c>
       <c r="K11">
         <v>8</v>
@@ -2303,19 +2303,19 @@
         <v>EUR</v>
       </c>
       <c r="F12">
-        <v>2.43</v>
+        <v>2.45</v>
       </c>
       <c r="G12">
-        <v>3.25</v>
+        <v>3.24</v>
       </c>
       <c r="H12" t="str">
         <v>A-</v>
       </c>
       <c r="I12">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J12" t="str">
-        <v>€42.25 Million</v>
+        <v>€42.28 Million</v>
       </c>
       <c r="K12">
         <v>9</v>
@@ -2341,7 +2341,7 @@
         <v>EUR</v>
       </c>
       <c r="F13">
-        <v>0.77</v>
+        <v>0.84</v>
       </c>
       <c r="G13">
         <v>2.63</v>
@@ -2350,10 +2350,10 @@
         <v>AA-</v>
       </c>
       <c r="I13">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J13" t="str">
-        <v>€599.62 Million</v>
+        <v>€599.70 Million</v>
       </c>
       <c r="K13">
         <v>8</v>
@@ -2379,7 +2379,7 @@
         <v>EUR</v>
       </c>
       <c r="F14">
-        <v>0.77</v>
+        <v>0.84</v>
       </c>
       <c r="G14">
         <v>2.63</v>
@@ -2388,10 +2388,10 @@
         <v>AA-</v>
       </c>
       <c r="I14">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J14" t="str">
-        <v>€599.62 Million</v>
+        <v>€599.70 Million</v>
       </c>
       <c r="K14">
         <v>8</v>

</xml_diff>